<commit_message>
PG-0S has been modified and two new examples have been added
</commit_message>
<xml_diff>
--- a/utilities/permutational_symmetry/Young_Tableaux.xlsx
+++ b/utilities/permutational_symmetry/Young_Tableaux.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nuedukz-my.sharepoint.com/personal/sergiy_bubin_nu_edu_kz/Documents/Temp/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/78a8521088551d44/code/new_git/ecgpack/utilities/permutational_symmetry/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="199" documentId="8_{84B59777-9BE7-4800-A167-BEE100C7FD5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A7C14DCD-6F9A-4BA1-8BD3-264F783C9B43}"/>
   <bookViews>
-    <workbookView xWindow="52" yWindow="218" windowWidth="24600" windowHeight="30615" xr2:uid="{93188771-0260-44D0-BD5C-6A8BDDDE7860}"/>
+    <workbookView xWindow="-120" yWindow="0" windowWidth="23280" windowHeight="25320" xr2:uid="{93188771-0260-44D0-BD5C-6A8BDDDE7860}"/>
   </bookViews>
   <sheets>
     <sheet name="Left-Down_scheme" sheetId="1" r:id="rId1"/>
@@ -692,20 +692,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22CA9807-4B80-43C0-A71E-424C5F39765A}">
   <dimension ref="A1:AA66"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.59765625" style="4" customWidth="1"/>
-    <col min="2" max="7" width="6.59765625" customWidth="1"/>
-    <col min="8" max="8" width="6.59765625" style="1" customWidth="1"/>
-    <col min="9" max="28" width="6.59765625" customWidth="1"/>
+    <col min="1" max="1" width="6.5546875" style="4" customWidth="1"/>
+    <col min="2" max="7" width="6.5546875" customWidth="1"/>
+    <col min="8" max="8" width="6.5546875" style="1" customWidth="1"/>
+    <col min="9" max="28" width="6.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
         <v>29</v>
       </c>
@@ -719,7 +719,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4">
         <v>3</v>
       </c>
@@ -737,20 +737,20 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="I4" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="I5" s="8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="H6" s="8"/>
     </row>
-    <row r="7" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C7" s="9" t="s">
         <v>2</v>
       </c>
@@ -761,7 +761,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
         <v>4</v>
       </c>
@@ -779,7 +779,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C9" s="5">
         <v>4</v>
       </c>
@@ -788,7 +788,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C10" s="8" t="s">
         <v>6</v>
       </c>
@@ -796,13 +796,13 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="I11" s="8" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="13" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="13" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4">
         <v>5</v>
       </c>
@@ -824,7 +824,7 @@
       <c r="P13" s="3"/>
       <c r="Q13" s="3"/>
     </row>
-    <row r="14" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C14" s="2">
         <v>2</v>
       </c>
@@ -849,7 +849,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C15" s="2">
         <v>4</v>
       </c>
@@ -869,7 +869,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C16" s="8" t="s">
         <v>6</v>
       </c>
@@ -886,7 +886,7 @@
       <c r="P16" s="8"/>
       <c r="Q16" s="8"/>
     </row>
-    <row r="17" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="I17" s="8" t="s">
         <v>10</v>
       </c>
@@ -894,13 +894,13 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="I18" s="1"/>
       <c r="O18" s="8" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4">
         <v>6</v>
       </c>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C20" s="2">
         <v>2</v>
       </c>
@@ -945,7 +945,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C21" s="2">
         <v>4</v>
       </c>
@@ -965,7 +965,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C22" s="2">
         <v>6</v>
       </c>
@@ -977,7 +977,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="23" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C23" s="8" t="s">
         <v>11</v>
       </c>
@@ -988,7 +988,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D24" s="8" t="s">
         <v>8</v>
       </c>
@@ -999,14 +999,14 @@
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="I25" s="1"/>
       <c r="O25" s="8" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="26" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="27" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="27" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="4">
         <v>7</v>
       </c>
@@ -1029,7 +1029,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="28" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C28" s="2">
         <v>2</v>
       </c>
@@ -1063,7 +1063,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C29" s="2">
         <v>4</v>
       </c>
@@ -1091,7 +1091,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="30" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C30" s="2">
         <v>6</v>
       </c>
@@ -1113,7 +1113,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C31" s="8" t="s">
         <v>11</v>
       </c>
@@ -1127,7 +1127,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D32" s="8" t="s">
         <v>23</v>
       </c>
@@ -1141,7 +1141,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="33" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="I33" s="1"/>
       <c r="J33" s="8" t="s">
         <v>8</v>
@@ -1153,14 +1153,14 @@
         <v>7</v>
       </c>
     </row>
-    <row r="34" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="I34" s="1"/>
       <c r="U34" s="8" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="35" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="36" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="36" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="4">
         <v>8</v>
       </c>
@@ -1183,7 +1183,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="37" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C37" s="2">
         <v>2</v>
       </c>
@@ -1217,7 +1217,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="38" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C38" s="2">
         <v>4</v>
       </c>
@@ -1245,7 +1245,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="39" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C39" s="2">
         <v>6</v>
       </c>
@@ -1267,7 +1267,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="40" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C40" s="2">
         <v>8</v>
       </c>
@@ -1281,7 +1281,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="41" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C41" s="8" t="s">
         <v>22</v>
       </c>
@@ -1295,7 +1295,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="42" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D42" s="8" t="s">
         <v>23</v>
       </c>
@@ -1309,7 +1309,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="43" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="I43" s="1"/>
       <c r="J43" s="8" t="s">
         <v>8</v>
@@ -1321,13 +1321,13 @@
         <v>8</v>
       </c>
     </row>
-    <row r="44" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="U44" s="8" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="45" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="46" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="46" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="4">
         <v>9</v>
       </c>
@@ -1353,7 +1353,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="47" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C47" s="2">
         <v>2</v>
       </c>
@@ -1396,7 +1396,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="48" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C48" s="2">
         <v>4</v>
       </c>
@@ -1433,7 +1433,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="49" spans="3:27" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="49" spans="3:27" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C49" s="2">
         <v>6</v>
       </c>
@@ -1465,7 +1465,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="50" spans="3:27" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="50" spans="3:27" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C50" s="2">
         <v>8</v>
       </c>
@@ -1492,7 +1492,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="51" spans="3:27" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="51" spans="3:27" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C51" s="8" t="s">
         <v>22</v>
       </c>
@@ -1509,7 +1509,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="52" spans="3:27" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="52" spans="3:27" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D52" s="8" t="s">
         <v>31</v>
       </c>
@@ -1526,7 +1526,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="53" spans="3:27" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="53" spans="3:27" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="J53" s="8" t="s">
         <v>23</v>
       </c>
@@ -1540,7 +1540,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="54" spans="3:27" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="54" spans="3:27" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="P54" s="8" t="s">
         <v>8</v>
       </c>
@@ -1548,26 +1548,26 @@
         <v>9</v>
       </c>
     </row>
-    <row r="55" spans="3:27" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="55" spans="3:27" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="U55" s="8" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="56" spans="3:27" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="56" spans="3:27" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="AA56" s="8" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="57" spans="3:27" ht="36" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="58" spans="3:27" ht="36" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="59" spans="3:27" ht="36" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="60" spans="3:27" ht="36" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="61" spans="3:27" ht="36" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="62" spans="3:27" ht="36" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="63" spans="3:27" ht="36" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="64" spans="3:27" ht="36" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="65" ht="36" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="66" ht="36" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="57" spans="3:27" ht="36" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="58" spans="3:27" ht="36" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="59" spans="3:27" ht="36" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="60" spans="3:27" ht="36" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="61" spans="3:27" ht="36" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="62" spans="3:27" ht="36" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="63" spans="3:27" ht="36" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="64" spans="3:27" ht="36" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="65" ht="36" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="66" ht="36" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>